<commit_message>
lots of flagging options
</commit_message>
<xml_diff>
--- a/HerculanoHouzel_etal_2015/HerculanoHouzel_etal_2015_Table3_snapshot.xlsx
+++ b/HerculanoHouzel_etal_2015/HerculanoHouzel_etal_2015_Table3_snapshot.xlsx
@@ -3766,8 +3766,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="acb3cbe4b9dee1876b3bbe7116f679b3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ca927c27970307cd175704f09b582c5c" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="66af2654134d243f62aac8e2b322f1d6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2bc3adf68671d86faa9c37249f400344" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
     <xsd:import namespace="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
     <xsd:element name="properties">
@@ -3790,6 +3790,7 @@
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -3859,6 +3860,11 @@
     <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="22" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="23" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -4028,20 +4034,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A4AF0D9-BCD8-43F2-8D33-2ED063C6CB9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67CF396A-2EC2-4809-9F39-5195BDE52EEB}"/>
 </file>
</xml_diff>